<commit_message>
add: yml file에 fetch_state_by_blog_name.py 추가
</commit_message>
<xml_diff>
--- a/upload/keywords.xlsx
+++ b/upload/keywords.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zasq1\python\fetch\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892D53ED-A961-49F8-97F1-800B6B80F4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7695198-345E-4495-AE61-E4A48E7F868A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0CCAFDB8-1330-457B-999A-F05A412A75AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$85</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,175 +39,196 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
-  <si>
-    <t>keyword</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+  <si>
+    <t>맨드로포즈</t>
+  </si>
+  <si>
+    <t>요로굿</t>
+  </si>
+  <si>
+    <t>인-칼슘앱솔브</t>
+  </si>
+  <si>
+    <t>블러드플로우케어</t>
+  </si>
+  <si>
+    <t>조인트리션뮤코</t>
+  </si>
+  <si>
+    <t>185커큐민</t>
+  </si>
+  <si>
+    <t>출환</t>
+  </si>
+  <si>
+    <t>오큘라레이드</t>
+  </si>
+  <si>
+    <t>헤모웰당</t>
+  </si>
+  <si>
+    <t>요레스</t>
+  </si>
+  <si>
+    <t>위이지케어</t>
+  </si>
+  <si>
+    <t>조인트리션</t>
+  </si>
+  <si>
+    <t>초기1이유식</t>
+  </si>
+  <si>
+    <t>조인트리션릴리버</t>
+  </si>
+  <si>
+    <t>유기농비타민D3코어</t>
+  </si>
+  <si>
+    <t>그로우뉴</t>
+  </si>
+  <si>
+    <t>파미로겐</t>
+  </si>
+  <si>
+    <t>모환</t>
+  </si>
+  <si>
+    <t>지니어스뉴</t>
+  </si>
+  <si>
+    <t>휴환</t>
+  </si>
+  <si>
+    <t>슬립밸런스</t>
+  </si>
+  <si>
+    <t>유기농멀티비타민&amp;미네랄코어</t>
+  </si>
+  <si>
+    <t>후기무른밥</t>
+  </si>
+  <si>
+    <t>흑본전탕</t>
+  </si>
+  <si>
+    <t>투데이D3</t>
+  </si>
+  <si>
+    <t>지니어스뉴드롭스</t>
+  </si>
+  <si>
+    <t>유기농비타민D3</t>
+  </si>
+  <si>
+    <t>에피베리어</t>
+  </si>
+  <si>
+    <t>후기1이유식</t>
+  </si>
+  <si>
+    <t>후기이유식</t>
+  </si>
+  <si>
+    <t>데이프로바</t>
+  </si>
+  <si>
+    <t>이트뮨</t>
+  </si>
+  <si>
+    <t>리버티엑스</t>
+  </si>
+  <si>
+    <t>메노믹스</t>
+  </si>
+  <si>
+    <t>지니어스뉴키즈</t>
+  </si>
+  <si>
+    <t>인칼슘앱솔브</t>
+  </si>
+  <si>
+    <t>과일&amp;치즈퓨레</t>
+  </si>
+  <si>
+    <t>리베티컬</t>
+  </si>
+  <si>
+    <t>흑보목</t>
+  </si>
+  <si>
+    <t>초기2이유식</t>
+  </si>
+  <si>
+    <t>준비기이유식</t>
+  </si>
+  <si>
+    <t>중기이유식</t>
+  </si>
+  <si>
+    <t>유아식</t>
+  </si>
+  <si>
+    <t>영양밥찬국</t>
+  </si>
+  <si>
+    <t>투데이디3밤</t>
+  </si>
+  <si>
+    <t>초기1초기2이유식</t>
+  </si>
+  <si>
+    <t>후기2이유식</t>
+  </si>
+  <si>
+    <t>이트뮨배도라지주스</t>
+  </si>
+  <si>
+    <t>유기농비타민3코어</t>
+  </si>
+  <si>
+    <t>포스앤드</t>
+  </si>
+  <si>
+    <t>블러드슈가케어</t>
+  </si>
+  <si>
+    <t>처음클레과일칩</t>
+  </si>
+  <si>
+    <t>초기이유식</t>
+  </si>
+  <si>
+    <t>글루코믹스</t>
+  </si>
+  <si>
+    <t>이유식</t>
+  </si>
+  <si>
+    <t>쑥쑥클레아이첫김</t>
+  </si>
+  <si>
+    <t>클레유기농그릭요거트</t>
+  </si>
+  <si>
+    <t>클레쌀떡뻥</t>
+  </si>
+  <si>
+    <t>수드티</t>
+  </si>
+  <si>
+    <t>리듀스앤드</t>
+  </si>
+  <si>
+    <t>런앤드</t>
+  </si>
+  <si>
+    <t>인칼슘앱솔브+</t>
+  </si>
+  <si>
+    <t>item</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>임산부에좋은차</t>
-  </si>
-  <si>
-    <t>입덧에좋은음식</t>
-  </si>
-  <si>
-    <t>입덧완화음식</t>
-  </si>
-  <si>
-    <t>입덧에좋은차</t>
-  </si>
-  <si>
-    <t>입덧할때음식</t>
-  </si>
-  <si>
-    <t>임산부입덧음식</t>
-  </si>
-  <si>
-    <t>입덧완화방법</t>
-  </si>
-  <si>
-    <t>입덧완화밴드</t>
-  </si>
-  <si>
-    <t>입덧완화차</t>
-  </si>
-  <si>
-    <t>입덧완화캔디</t>
-  </si>
-  <si>
-    <t>입덧캔디</t>
-  </si>
-  <si>
-    <t>입덧심할때</t>
-  </si>
-  <si>
-    <t>임산부입덧약</t>
-  </si>
-  <si>
-    <t>입덧완화</t>
-  </si>
-  <si>
-    <t>입덧수액</t>
-  </si>
-  <si>
-    <t>입덧토</t>
-  </si>
-  <si>
-    <t>입덧약부작용</t>
-  </si>
-  <si>
-    <t>입덧약</t>
-  </si>
-  <si>
-    <t>입덧약효과</t>
-  </si>
-  <si>
-    <t>입덧약처방</t>
-  </si>
-  <si>
-    <t>입덧약실비</t>
-  </si>
-  <si>
-    <t>입덧약성분</t>
-  </si>
-  <si>
-    <t>입덧약종류</t>
-  </si>
-  <si>
-    <t>입덧약약국</t>
-  </si>
-  <si>
-    <t>입덧약효과시간</t>
-  </si>
-  <si>
-    <t>입덧약가격</t>
-  </si>
-  <si>
-    <t>입덧약디클렉틴</t>
-  </si>
-  <si>
-    <t>입덧약두통</t>
-  </si>
-  <si>
-    <t>임신입덧시기</t>
-  </si>
-  <si>
-    <t>입덧증상</t>
-  </si>
-  <si>
-    <t>입덧음식</t>
-  </si>
-  <si>
-    <t>입덧이유</t>
-  </si>
-  <si>
-    <t>입덧시기</t>
-  </si>
-  <si>
-    <t>입덧시작시기</t>
-  </si>
-  <si>
-    <t>입덧끝나는시기</t>
-  </si>
-  <si>
-    <t>루이보스차</t>
-  </si>
-  <si>
-    <t>임산부에게좋은차</t>
-  </si>
-  <si>
-    <t>임산부에게좋은음식</t>
-  </si>
-  <si>
-    <t>임산부에게좋은과일</t>
-  </si>
-  <si>
-    <t>임산부음료</t>
-  </si>
-  <si>
-    <t>임산부음료수</t>
-  </si>
-  <si>
-    <t>산모음식</t>
-  </si>
-  <si>
-    <t>임산부음식</t>
-  </si>
-  <si>
-    <t>산모에게좋은음식</t>
-  </si>
-  <si>
-    <t>산모영양제</t>
-  </si>
-  <si>
-    <t>산모간식</t>
-  </si>
-  <si>
-    <t>산모식단</t>
-  </si>
-  <si>
-    <t>산모반찬</t>
-  </si>
-  <si>
-    <t>임산부루이보스티</t>
-  </si>
-  <si>
-    <t>임산부루이보스</t>
-  </si>
-  <si>
-    <t>임산부로이보스차</t>
-  </si>
-  <si>
-    <t>루이보스티효능</t>
-  </si>
-  <si>
-    <t>루이보스카페인</t>
-  </si>
-  <si>
-    <t>루이보스효능</t>
-  </si>
-  <si>
-    <t>임신축하선물</t>
   </si>
 </sst>
 </file>
@@ -600,290 +624,332 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{337A0CED-F72F-4749-808E-001C837951DF}">
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>